<commit_message>
feat: update Hoenn routes and generate documentation spreadsheets
- Scales main route encounters from level 1 up to level 70 (Pokemon League).
- Adds and inserts 'Advanced Starter Sanctuary' into the A-chain of extra challenges.
- Smoothly scales extra challenges up to level 100, and assigns fixed high levels to Legendaries/Mythicals (e.g. Deoxys 120, Jirachi 120).
- Distributes requested missing Hoenn Pokémon across logical routes based on typings.
- Generates `3_Hoenn_Data.xlsx` and `Region3Spots.xlsx` mapping all game locations, spawns, unlock chains, and obtainability.

Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Region3Spots.xlsx
+++ b/Region3Spots.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C56"/>
+  <dimension ref="A1:C57"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -888,10 +888,10 @@
         <v>Extra Challenge A 3</v>
       </c>
       <c r="B45" t="str">
-        <v>Daycare Special Spot</v>
+        <v>Advanced Starter Sanctuary</v>
       </c>
       <c r="C45">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="46">
@@ -899,7 +899,7 @@
         <v>Extra Challenge A 4</v>
       </c>
       <c r="B46" t="str">
-        <v>Battle Frontier Facility</v>
+        <v>Daycare Special Spot</v>
       </c>
       <c r="C46">
         <v>0</v>
@@ -910,7 +910,7 @@
         <v>Extra Challenge A 5</v>
       </c>
       <c r="B47" t="str">
-        <v>Weather Climax Cave</v>
+        <v>Battle Frontier Facility</v>
       </c>
       <c r="C47">
         <v>0</v>
@@ -918,10 +918,10 @@
     </row>
     <row r="48">
       <c r="A48" t="str">
-        <v>Extra Challenge B 1</v>
+        <v>Extra Challenge A 6</v>
       </c>
       <c r="B48" t="str">
-        <v>Trick House</v>
+        <v>Weather Climax Cave</v>
       </c>
       <c r="C48">
         <v>0</v>
@@ -929,10 +929,10 @@
     </row>
     <row r="49">
       <c r="A49" t="str">
-        <v>Extra Challenge B 2</v>
+        <v>Extra Challenge B 1</v>
       </c>
       <c r="B49" t="str">
-        <v>Rustboro Fossil Lab</v>
+        <v>Trick House</v>
       </c>
       <c r="C49">
         <v>0</v>
@@ -940,10 +940,10 @@
     </row>
     <row r="50">
       <c r="A50" t="str">
-        <v>Extra Challenge B 3</v>
+        <v>Extra Challenge B 2</v>
       </c>
       <c r="B50" t="str">
-        <v>Abandoned Ship</v>
+        <v>Rustboro Fossil Lab</v>
       </c>
       <c r="C50">
         <v>0</v>
@@ -951,10 +951,10 @@
     </row>
     <row r="51">
       <c r="A51" t="str">
-        <v>Extra Challenge B 4</v>
+        <v>Extra Challenge B 3</v>
       </c>
       <c r="B51" t="str">
-        <v>Enemy Hideout</v>
+        <v>Abandoned Ship</v>
       </c>
       <c r="C51">
         <v>0</v>
@@ -962,10 +962,10 @@
     </row>
     <row r="52">
       <c r="A52" t="str">
-        <v>Extra Challenge B 5</v>
+        <v>Extra Challenge B 4</v>
       </c>
       <c r="B52" t="str">
-        <v>Sealed Chamber</v>
+        <v>Enemy Hideout</v>
       </c>
       <c r="C52">
         <v>0</v>
@@ -973,10 +973,10 @@
     </row>
     <row r="53">
       <c r="A53" t="str">
-        <v>Extra Challenge B 6</v>
+        <v>Extra Challenge B 5</v>
       </c>
       <c r="B53" t="str">
-        <v>Ancient Ruins</v>
+        <v>Sealed Chamber</v>
       </c>
       <c r="C53">
         <v>0</v>
@@ -984,10 +984,10 @@
     </row>
     <row r="54">
       <c r="A54" t="str">
-        <v>Extra Challenge (Roaming)</v>
+        <v>Extra Challenge B 6</v>
       </c>
       <c r="B54" t="str">
-        <v>Roaming Hoenn Skies</v>
+        <v>Ancient Ruins</v>
       </c>
       <c r="C54">
         <v>0</v>
@@ -995,10 +995,10 @@
     </row>
     <row r="55">
       <c r="A55" t="str">
-        <v>Key to Nebula Fissure Challenge</v>
+        <v>Extra Challenge (Roaming)</v>
       </c>
       <c r="B55" t="str">
-        <v>Key to Nebula Fissure Challenge</v>
+        <v>Roaming Hoenn Skies</v>
       </c>
       <c r="C55">
         <v>0</v>
@@ -1006,18 +1006,29 @@
     </row>
     <row r="56">
       <c r="A56" t="str">
+        <v>Key to Nebula Fissure Challenge</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Key to Nebula Fissure Challenge</v>
+      </c>
+      <c r="C56">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
         <v>Nebula Fissure Challenge</v>
       </c>
-      <c r="B56" t="str">
+      <c r="B57" t="str">
         <v>Nebula Fissure</v>
       </c>
-      <c r="C56">
+      <c r="C57">
         <v>0</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C56"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C57"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>